<commit_message>
Fix: Single login fixed
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MobileAutomation\Smartschool_parent\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56ACEB50-164C-4FAE-A740-FF4BC9365746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32AE24B0-8A91-41A7-99BA-F6D69172C76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="39">
   <si>
     <t>TestCase</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>TC08_AlreadyAdded</t>
+  </si>
+  <si>
+    <t>TC03_3rd Mid Term</t>
+  </si>
+  <si>
+    <t>3rd Mid Term</t>
   </si>
 </sst>
 </file>
@@ -604,7 +610,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.81640625" bestFit="1" customWidth="1"/>
@@ -627,9 +633,6 @@
       <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
       <c r="C2" t="s">
         <v>16</v>
       </c>
@@ -643,6 +646,17 @@
       </c>
       <c r="C3" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: functional check completed
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MobileAutomation\Smartschool_parent\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32AE24B0-8A91-41A7-99BA-F6D69172C76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3164971E-EC58-4DDE-8EDB-CCD9A9576FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="41">
   <si>
     <t>TestCase</t>
   </si>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>3rd Mid Term</t>
+  </si>
+  <si>
+    <t>TC06_Parent2Login</t>
+  </si>
+  <si>
+    <t>MYST00590</t>
   </si>
 </sst>
 </file>
@@ -205,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -215,6 +221,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.26953125" bestFit="1" customWidth="1"/>
@@ -601,6 +608,17 @@
       </c>
       <c r="C6" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7">
+        <v>12012009</v>
       </c>
     </row>
   </sheetData>

</xml_diff>